<commit_message>
fix template for trans
</commit_message>
<xml_diff>
--- a/templates/barrisol_inv.xlsx
+++ b/templates/barrisol_inv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snigdhagoel/Documents/Vibrant Technik/vibrant-technik/barrisol-calculator/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DCE7F73-0F18-CD4B-827C-F9E03F507637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2980FADC-2D54-B440-9C7D-2378E7405AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15940" xr2:uid="{05935AE4-5CBA-6546-A82B-83CF6BB7C317}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15940" activeTab="1" xr2:uid="{05935AE4-5CBA-6546-A82B-83CF6BB7C317}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -888,6 +888,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -900,8 +902,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1254,33 +1254,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="2" customFormat="1" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="10"/>
-      <c r="B1" s="10"/>
-      <c r="C1" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
+      <c r="A1" s="12"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
       <c r="L1" s="1"/>
     </row>
     <row r="2" spans="1:12" s="2" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" s="2" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
@@ -2192,7 +2192,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4997BC04-D872-224A-BF31-FD022CCCA4C3}">
           <x14:formula1>
-            <xm:f>ACCESSORIES!$A$110:$A$116</xm:f>
+            <xm:f>ACCESSORIES!$A$98:$A$116</xm:f>
           </x14:formula1>
           <xm:sqref>B6</xm:sqref>
         </x14:dataValidation>
@@ -2452,7 +2452,7 @@
       </c>
     </row>
     <row r="28" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="11" t="s">
         <v>231</v>
       </c>
       <c r="B28" s="6" t="s">
@@ -2460,7 +2460,7 @@
       </c>
     </row>
     <row r="29" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="11" t="s">
         <v>233</v>
       </c>
       <c r="B29" s="6" t="s">
@@ -2660,7 +2660,7 @@
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" s="14" t="s">
+      <c r="A54" s="10" t="s">
         <v>235</v>
       </c>
       <c r="B54" s="6" t="s">
@@ -2668,7 +2668,7 @@
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" s="14" t="s">
+      <c r="A55" s="10" t="s">
         <v>237</v>
       </c>
       <c r="B55" s="6" t="s">

</xml_diff>